<commit_message>
Added enum to map point types between template and BAC0.
</commit_message>
<xml_diff>
--- a/tools/templates/point_template.xlsx
+++ b/tools/templates/point_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/d36616b/Documents/git/integrated-automation/nexuscon-2025/tools/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{525683FD-911C-2F4D-BBFB-1AD0D488C086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{532408DC-387D-D34A-88D3-A45C8D22E1B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20300" yWindow="-28300" windowWidth="34400" windowHeight="28300" xr2:uid="{1DAAB171-EED9-CD41-A923-E922B19884F4}"/>
+    <workbookView xWindow="-20280" yWindow="-28300" windowWidth="34400" windowHeight="28300" xr2:uid="{1DAAB171-EED9-CD41-A923-E922B19884F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Switch" sheetId="1" r:id="rId1"/>
@@ -119,7 +119,7 @@
     <t>Physical switch to toggle on/off connected LED</t>
   </si>
   <si>
-    <t>Test LED</t>
+    <t>LED that will toggle on/of with a physical switch</t>
   </si>
 </sst>
 </file>
@@ -832,7 +832,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>24</v>
       </c>

</xml_diff>

<commit_message>
Split out modules from the template handler.
</commit_message>
<xml_diff>
--- a/tools/templates/point_template.xlsx
+++ b/tools/templates/point_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/d36616b/Documents/git/integrated-automation/nexuscon-2025/tools/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{532408DC-387D-D34A-88D3-A45C8D22E1B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9381E500-B78C-0A45-9EA3-5E0425268CD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20280" yWindow="-28300" windowWidth="34400" windowHeight="28300" xr2:uid="{1DAAB171-EED9-CD41-A923-E922B19884F4}"/>
   </bookViews>
@@ -98,18 +98,12 @@
     <t>AO</t>
   </si>
   <si>
-    <t>%</t>
-  </si>
-  <si>
     <t>BI</t>
   </si>
   <si>
     <t>Boolean</t>
   </si>
   <si>
-    <t>FALSE,TRUE</t>
-  </si>
-  <si>
     <t>LEDOutput</t>
   </si>
   <si>
@@ -120,6 +114,12 @@
   </si>
   <si>
     <t>LED that will toggle on/of with a physical switch</t>
+  </si>
+  <si>
+    <t>PERCENT</t>
+  </si>
+  <si>
+    <t>BOOLEAN</t>
   </si>
 </sst>
 </file>
@@ -834,10 +834,10 @@
     </row>
     <row r="2" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>13</v>
@@ -849,7 +849,7 @@
         <v>14</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G2" s="2">
         <v>1</v>
@@ -875,22 +875,22 @@
     </row>
     <row r="3" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="F3" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G3" s="2">
         <v>1</v>

</xml_diff>